<commit_message>
Update benchmark workload to v1.0.14
</commit_message>
<xml_diff>
--- a/config/hw_sw_info_commands.xlsx
+++ b/config/hw_sw_info_commands.xlsx
@@ -1,2850 +1,3252 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E105"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Save Sequence</t>
+          <t>Save Sequence</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vendor</t>
+          <t>Vendor</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Info Domain</t>
+          <t>Info Domain</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Command</t>
+          <t>Command</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Description</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">101</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">date</t>
+          <t>date</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current Date and Time</t>
+          <t>Current Date and Time</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">102</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hostnamectl</t>
+          <t>hostnamectl</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hostname &amp; System Identity (VM/Host Details)</t>
+          <t>Hostname &amp; System Identity (VM/Host Details)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">103</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">lscpu | grep -E "Model name|Socket|Core|Thread|CPU\(s\)|MHz"</t>
+          <t>lscpu | grep -E "Model name|Socket|Core|Thread|CPU\(s\)|MHz"</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPU Model &amp; Core Count</t>
+          <t>CPU Model &amp; Core Count</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">104</t>
+          <t>104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">numactl --hardware</t>
+          <t>numactl --hardware</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUMA Topology &amp; Memory Layout</t>
+          <t>NUMA Topology &amp; Memory Layout</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">105</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">lsmem</t>
+          <t>lsmem</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">System Memory Total</t>
+          <t>System Memory Total</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">106</t>
+          <t>106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">free -h</t>
+          <t>free -h</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Memory (RAM)</t>
+          <t>Memory (RAM)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">107</t>
+          <t>107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">dmidecode -t memory | grep Size</t>
+          <t>dmidecode -t memory | grep Size</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Physical Memory Module Sizes</t>
+          <t>Physical Memory Module Sizes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">108</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">df -h</t>
+          <t>df -h</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Disk usage</t>
+          <t>Disk usage</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">109</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">lsblk -o NAME,SIZE,TYPE,MOUNTPOINT</t>
+          <t>lsblk -o NAME,SIZE,TYPE,MOUNTPOINT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Block Devices &amp; Mount Points</t>
+          <t>Block Devices &amp; Mount Points</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">110</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">dmidecode -t system | sed -n '/System Information/,/Family:/p'</t>
+          <t>dmidecode -t system | sed -n '/System Information/,/Family:/p'</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">System Hardware Info (Manufacturer, Product, UUID)</t>
+          <t>System Hardware Info (Manufacturer, Product, UUID)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci</t>
+          <t>lspci</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCI Device List</t>
+          <t>PCI Device List</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">112</t>
+          <t>112</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">lscpu</t>
+          <t>lscpu</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPU Architecture and Cache Info</t>
+          <t>CPU Architecture and Cache Info</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">113</t>
+          <t>113</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">ip addr show</t>
+          <t>ip addr show</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Network Interface Configuration</t>
+          <t>Network Interface Configuration</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">114</t>
+          <t>114</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">lsmod</t>
+          <t>lsmod</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loaded Kernel Modules</t>
+          <t>Loaded Kernel Modules</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">115</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">cat /proc/cpuinfo | head -19</t>
+          <t>cat /proc/cpuinfo | head -19</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPU Details (long)</t>
+          <t>CPU Details (long)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">116</t>
+          <t>116</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci | grep -i accelerator</t>
+          <t>lspci | grep -i accelerator</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Bus Address and Device ID</t>
+          <t>AMD GPU Bus Address and Device ID</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">117</t>
+          <t>117</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocminfo | grep gfx</t>
+          <t>rocminfo | grep gfx</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Architecture IDs (gfx)</t>
+          <t>AMD GPU Architecture IDs (gfx)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">118</t>
+          <t>118</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocm-smi --showmeminfo vram</t>
+          <t>amd-smi static --vram</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Details (Model, VRAM)</t>
+          <t>AMD GPU Details (Model, VRAM)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">119</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocm-smi --showproductname</t>
+          <t>amd-smi static --asic</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Product SKU and Identification</t>
+          <t>AMD GPU Product SKU and Identification</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">120</t>
+          <t>120</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -d 1002: | grep -E 'AMD|LnkCap:|LnkSta:|Region'</t>
+          <t>lspci -vv -d 1002: | grep -E 'AMD|LnkCap:|LnkSta:|Region'</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU PCIe Link &amp; Memory Regions</t>
+          <t>AMD GPU PCIe Link &amp; Memory Regions</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">121</t>
+          <t>121</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocm-smi</t>
+          <t>amd-smi metric</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Live Telemetry (Temp, Power, Clocks)</t>
+          <t>AMD GPU Live Telemetry (Temp, Power, Clocks)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">122</t>
+          <t>122</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -d 1002:</t>
+          <t>lspci -vv -d 1002:</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Full GPU PCI Details</t>
+          <t>AMD Full GPU PCI Details</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">123</t>
+          <t>123</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">amd-smi static | head -30</t>
+          <t>amd-smi static | head -30</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Hardware Identity</t>
+          <t>AMD GPU Hardware Identity</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">124</t>
+          <t>124</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocminfo | grep Name</t>
+          <t>rocminfo | grep Name</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU/CPU Agent Names (ROCm Info)</t>
+          <t>AMD GPU/CPU Agent Names (ROCm Info)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">125</t>
+          <t>125</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">amd-smi</t>
+          <t>amd-smi</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU Overview and Status</t>
+          <t>AMD GPU Overview and Status</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">126</t>
+          <t>126</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">dmesg | grep -Ei 'amdgpu|xgmi|kfd|rocm'</t>
+          <t>dmesg | grep -Ei 'amdgpu|xgmi|kfd|rocm'</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Kernel Boot Log - AMD/GPU Messages</t>
+          <t>AMD Kernel Boot Log - AMD/GPU Messages</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">127</t>
+          <t>127</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -s $(lspci | grep -i accelerator | awk '{print $1}' | head -1)</t>
+          <t>lspci -vv -s $(lspci | grep -i accelerator | awk '{print $1}' | head -1)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD GPU PCI Config (Link, BARs, Driver Binding)</t>
+          <t>AMD GPU PCI Config (Link, BARs, Driver Binding)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">128</t>
+          <t>128</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi --query-gpu=name,pci.bus_id --format=csv</t>
+          <t>nvidia-smi --query-gpu=name,pci.bus_id --format=csv</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU Agent Names</t>
+          <t>nVidia GPU Agent Names</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">129</t>
+          <t>129</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci | grep -i nvidia</t>
+          <t>lspci | grep -i nvidia</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU Bus Address and Device ID</t>
+          <t>nVidia GPU Bus Address and Device ID</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">130</t>
+          <t>130</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi --query-gpu=memory.total --format=csv</t>
+          <t>nvidia-smi --query-gpu=memory.total --format=csv</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU Details (VRAM)</t>
+          <t>nVidia GPU Details (VRAM)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">131</t>
+          <t>131</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -d 10de: | grep -E 'NVIDIA|LnkCap:|LnkSta:|Region'</t>
+          <t>lspci -vv -d 10de: | grep -E 'NVIDIA|LnkCap:|LnkSta:|Region'</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU PCIe Link &amp; Memory Regions</t>
+          <t>nVidia GPU PCIe Link &amp; Memory Regions</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">132</t>
+          <t>132</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi</t>
+          <t>nvidia-smi</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU Live Telemetry (Temp, Power, Clocks)</t>
+          <t>nVidia GPU Live Telemetry (Temp, Power, Clocks)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">133</t>
+          <t>133</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -d 10de:</t>
+          <t>lspci -vv -d 10de:</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia Full GPU PCI details (long)</t>
+          <t>nVidia Full GPU PCI details (long)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">134</t>
+          <t>134</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi -q | head -30</t>
+          <t>nvidia-smi -q | head -30</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU hardware identity</t>
+          <t>nVidia GPU hardware identity</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">135</t>
+          <t>135</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi --query-gpu=compute_cap --format=csv</t>
+          <t>nvidia-smi --query-gpu=compute_cap --format=csv</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia GPU compute capability (9.0=sm_90)</t>
+          <t>nVidia GPU compute capability (9.0=sm_90)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">136</t>
+          <t>136</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W libnvidia-ml1</t>
+          <t>dpkg-query -W libnvidia-ml1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia NVML library version</t>
+          <t>nVidia NVML library version</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">137</t>
+          <t>137</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">dmesg | grep -Ei 'nvidia|nvrm|xid'</t>
+          <t>dmesg | grep -Ei 'nvidia|nvrm|xid'</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia kernel messages (Runpod permission fail)</t>
+          <t>nVidia kernel messages (Runpod permission fail)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">138</t>
+          <t>138</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">hardware</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">lspci -vv -s $(nvidia-smi --query-gpu=pci.bus_id --format=csv,noheader)</t>
+          <t>lspci -vv -s $(nvidia-smi --query-gpu=pci.bus_id --format=csv,noheader)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia PCI config (BARSs, Driver Binding)</t>
+          <t>nVidia PCI config (BARSs, Driver Binding)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">139</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">lsb_release -a</t>
+          <t>lsb_release -a</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">OS version &amp; Ubuntu release</t>
+          <t>OS version &amp; Ubuntu release</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">140</t>
+          <t>140</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">uname -a</t>
+          <t>uname -a</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linux Kernel Version</t>
+          <t>Linux Kernel Version</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">141</t>
+          <t>141</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">dkms --version</t>
+          <t>dkms --version</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kernel Modules (DKMS) Version</t>
+          <t>Kernel Modules (DKMS) Version</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">142</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">dkms status</t>
+          <t>dkms status</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kernel Modules (DKMS) Status</t>
+          <t>Kernel Modules (DKMS) Status</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">143</t>
+          <t>143</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 --version</t>
+          <t>python3 --version</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Python version</t>
+          <t>Python version</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">144</t>
+          <t>144</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import torch; print(torch.__version__)"</t>
+          <t>python3 -c "import torch; print(torch.__version__)"</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">PyTorch Version (generic)</t>
+          <t>PyTorch Version (generic)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">145</t>
+          <t>145</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W libnuma1</t>
+          <t>dpkg-query -W libnuma1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUMA library (libuma) version</t>
+          <t>NUMA library (libuma) version</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">146</t>
+          <t>146</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import torchvision; print(torchvision.__version__)"</t>
+          <t>python3 -c "import torchvision; print(torchvision.__version__)"</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">TorchVision version</t>
+          <t>TorchVision version</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">147</t>
+          <t>147</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -m pip show torchbench | grep -E '^Name:|^Version:|^Summary:'</t>
+          <t>python3 -m pip show torchbench | grep -E '^Name:|^Version:|^Summary:'</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TorchBench package info</t>
+          <t>TorchBench package info</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">148</t>
+          <t>148</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">pytest --version</t>
+          <t>pytest --version</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pytest version</t>
+          <t>Pytest version</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">149</t>
+          <t>149</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">numactl --version</t>
+          <t>numactl --version</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUMA Control Tool (numactl) Version</t>
+          <t>NUMA Control Tool (numactl) Version</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">150</t>
+          <t>150</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import triton; print(triton.__version__)"</t>
+          <t>python3 -c "import triton; print(triton.__version__)"</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Triton compiler version</t>
+          <t>Triton compiler version</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">151</t>
+          <t>151</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">clang --version | head -1</t>
+          <t>clang --version | head -1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clang compiler version</t>
+          <t>Clang compiler version</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">152</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">gcc --version  | head -1</t>
+          <t>gcc --version  | head -1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">GCC compiler version</t>
+          <t>GCC compiler version</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">153</t>
+          <t>153</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">g++ --version | head -1</t>
+          <t>g++ --version | head -1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">G++ compiler version</t>
+          <t>G++ compiler version</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">154</t>
+          <t>154</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">cmake --version | head -1</t>
+          <t>cmake --version | head -1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMake version</t>
+          <t>CMake version</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">155</t>
+          <t>155</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">make --version | head -2</t>
+          <t>make --version | head -2</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Make utility version</t>
+          <t>Make utility version</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">156</t>
+          <t>156</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">bash --version | head -1</t>
+          <t>bash --version | head -1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bash version</t>
+          <t>Bash version</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">157</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">mpirun --version | head -1</t>
+          <t>mpirun --version | head -1</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPI runtime (mpirun) version</t>
+          <t>MPI runtime (mpirun) version</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">158</t>
+          <t>158</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">fio --version</t>
+          <t>fio --version</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIO benchmark version</t>
+          <t>FIO benchmark version</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">159</t>
+          <t>159</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvme version</t>
+          <t>nvme version</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">NVMe CLI version</t>
+          <t>NVMe CLI version</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">160</t>
+          <t>160</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import sglang; print(sglang.__version__)"</t>
+          <t>python3 -c "import sglang; print(sglang.__version__)"</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">SGLang version</t>
+          <t>SGLang version</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">161</t>
+          <t>161</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">iperf3 --version | head -1</t>
+          <t>iperf3 --version | head -1</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPerf3 version</t>
+          <t>iPerf3 version</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">162</t>
+          <t>162</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import vllm; print(vllm.__version__)"</t>
+          <t>python3 -c "import vllm; print(vllm.__version__)"</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">vLLM version</t>
+          <t>vLLM version</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">163</t>
+          <t>163</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import jax; print(jax.__version__)"</t>
+          <t>python3 -c "import jax; print(jax.__version__)"</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">JAX version</t>
+          <t>JAX version</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">164</t>
+          <t>164</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import jaxlib; print(jaxlib.__version__)"</t>
+          <t>python3 -c "import jaxlib; print(jaxlib.__version__)"</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">JAXlib version</t>
+          <t>JAXlib version</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">165</t>
+          <t>165</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W libaio1t64</t>
+          <t>dpkg-query -W libaio1t64</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">libaio (Linux AIO library) version</t>
+          <t>libaio (Linux AIO library) version</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">166</t>
+          <t>166</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import faiss; print(faiss.__version__)"</t>
+          <t>python3 -c "import faiss; print(faiss.__version__)"</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAISS version</t>
+          <t>FAISS version</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">167</t>
+          <t>167</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import diffusers; print(diffusers.__version__)"</t>
+          <t>python3 -c "import diffusers; print(diffusers.__version__)"</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diffusers library version</t>
+          <t>Diffusers library version</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">168</t>
+          <t>168</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg -l | grep -i lmbench</t>
+          <t>dpkg -l | grep -i lmbench</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">lmbench package version</t>
+          <t>lmbench package version</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">169</t>
+          <t>169</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">gcc -fopenmp -dM -E - &lt; /dev/null | grep _OPENMP</t>
+          <t>gcc -fopenmp -dM -E - &lt; /dev/null | grep _OPENMP</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">OpenMP version</t>
+          <t>OpenMP version</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">170</t>
+          <t>170</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">pip show llama-index | grep Version</t>
+          <t>pip show llama-index | grep Version</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">LlamaIndex version</t>
+          <t>LlamaIndex version</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">171</t>
+          <t>171</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">huggingface-cli scan-cache | grep -i mistra</t>
+          <t>huggingface-cli scan-cache | grep -i mistra</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mistral model revision</t>
+          <t>Mistral model revision</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">172</t>
+          <t>172</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import yaml; print(yaml.__version__)"</t>
+          <t>python3 -c "import yaml; print(yaml.__version__)"</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">PyYAML version</t>
+          <t>PyYAML version</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">173</t>
+          <t>173</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">sqlite3 --version</t>
+          <t>sqlite3 --version</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">SQLite version</t>
+          <t>SQLite version</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">174</t>
+          <t>174</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">perf --version</t>
+          <t>perf --version</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perf tool (Linux perf) version</t>
+          <t>Perf tool (Linux perf) version</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">175</t>
+          <t>175</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">stress-ng --version</t>
+          <t>stress-ng --version</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">stress-ng version</t>
+          <t>stress-ng version</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">176</t>
+          <t>176</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">bc --version | head -1</t>
+          <t>bc --version | head -1</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">BC calculator (bc) Version</t>
+          <t>BC calculator (bc) Version</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">177</t>
+          <t>177</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD, nVidia</t>
+          <t>AMD, nVidia</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t xml:space="preserve">jq --version</t>
+          <t>jq --version</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">JQ (jq) Version</t>
+          <t>JQ (jq) Version</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">178</t>
+          <t>178</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W rocm-core</t>
+          <t>dpkg-query -W amdrocm-base10.1</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Installed ROCm version</t>
+          <t>AMD Installed ROCm version (amdrocm-base10.1)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">179</t>
+          <t>179</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">amd-smi version</t>
+          <t>amd-smi version</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD SMI Tool &amp; Library Versions</t>
+          <t>AMD SMI Tool &amp; Library Versions</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">180</t>
+          <t>180</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">hipcc --version</t>
+          <t>hipcc --version</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD HIP Compiler Version</t>
+          <t>AMD HIP Compiler Version</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">181</t>
+          <t>181</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import torch; print(torch.version.hip)"</t>
+          <t>python3 -c "import torch; print(torch.version.hip)"</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD PyTorch HIP Version (AMD GPU)</t>
+          <t>AMD PyTorch HIP Version (AMD GPU)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">182</t>
+          <t>182</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W miopen-hip</t>
+          <t>dpkg-query -W amdrocm-dnn-host10.1</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD MIOpen HIP version</t>
+          <t>AMD MIOpen version (amdrocm-dnn-host10.1)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">183</t>
+          <t>183</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocm-smi --version</t>
+          <t>amd-smi firmware</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD ROCm SMI version</t>
+          <t>AMD GPU Firmware Versions (AMD SMI)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">184</t>
+          <t>184</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W rccl</t>
+          <t>dpkg-query -W amdrocm-rccl-host10.1</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD RCCL version</t>
+          <t>AMD RCCL version (amdrocm-rccl-host10.1)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">185</t>
+          <t>185</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W rocblas</t>
+          <t>dpkg-query -W amdrocm-blas10.1</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Installed rocBLAS version</t>
+          <t>AMD Installed rocBLAS version (amdrocm-blas10.1)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">186</t>
+          <t>186</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W rocsolver</t>
+          <t>dpkg-query -W amdrocm-solver-host10.1</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD rocSOLVER version</t>
+          <t>AMD rocSOLVER version (amdrocm-solver-host10.1)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">187</t>
+          <t>187</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t xml:space="preserve">rochpl --version</t>
+          <t>rochpl --version</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD rocHPL version</t>
+          <t>AMD rocHPL version</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">188</t>
+          <t>188</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">echo "RVS Version: $(/opt/rocm/bin/rvs --version)"</t>
+          <t>echo "RVS Version: $(rvs --version)"</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD ROCm Validation Suite version</t>
+          <t>AMD ROCm Validation Suite version</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">189</t>
+          <t>189</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg -l | egrep -i '^(ii)\s+(amdgpu-install |amd-smi-lib |hipblas |hipblaslt |hipcc |hipfft |hiprand |hip-runtime-amd |hipsolver |hipsparse |hiptensor |hsa-rocr |libgl1-amdgpu-mesa-dri:amd64 |llvm-amdgpu |miopen-hip |opencl-rocm |rccl |rocblas |rocblaslt |rocfft |rocm-core |rocm-llvm |rocm-validation-suite |rocprim-dev |rocprofiler |rocrand |rocsolver |rocsparse |rocthrust-dev |rocwmma-dev )'</t>
+          <t>dpkg -l | egrep -i '^ii\s+(amdrocm|amdgpu)'</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Installed ROCm &amp; AMD Packages List</t>
+          <t>AMD Installed ROCm &amp; AMD Packages List</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">190</t>
+          <t>190</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">hipconfig  --full</t>
+          <t>hipconfig  --full</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD HIP / ROCm Configuration Details</t>
+          <t>AMD HIP / ROCm Configuration Details</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">191</t>
+          <t>191</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">apt list --installed | grep rocm</t>
+          <t>apt list --installed | grep rocm</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD Installed ROCm Packages</t>
+          <t>AMD Installed ROCm Packages</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">192</t>
+          <t>192</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD-only</t>
+          <t>AMD-only</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">rocminfo</t>
+          <t>rocminfo</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD ROCm HSA Runtime Details</t>
+          <t>AMD ROCm HSA Runtime Details</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">193</t>
+          <t>193</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvcc --version</t>
+          <t>nvcc --version</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia CUDA Toolkit and Compiler Details</t>
+          <t>nVidia CUDA Toolkit and Compiler Details</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">194</t>
+          <t>194</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi --version</t>
+          <t>nvidia-smi --version</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia SMI Tool &amp; NVML Library Versions</t>
+          <t>nVidia SMI Tool &amp; NVML Library Versions</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">195</t>
+          <t>195</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W cuda-toolkit</t>
+          <t>dpkg-query -W cuda-toolkit</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia Installed CUDA toolkit</t>
+          <t>nVidia Installed CUDA toolkit</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">196</t>
+          <t>196</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W "libcublas*"</t>
+          <t>dpkg-query -W "libcublas*"</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia Installed cuBLAS library</t>
+          <t>nVidia Installed cuBLAS library</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">197</t>
+          <t>197</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 -c "import torch; print(torch.version.cuda)"</t>
+          <t>python3 -c "import torch; print(torch.version.cuda)"</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia PyTorch CUDA version</t>
+          <t>nVidia PyTorch CUDA version</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">198</t>
+          <t>198</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W libcudnn\*</t>
+          <t>dpkg-query -W libcudnn\*</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia cuDNN version</t>
+          <t>nVidia cuDNN version</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">199</t>
+          <t>199</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W libnccl\*</t>
+          <t>dpkg-query -W libnccl\*</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia NCCL version</t>
+          <t>nVidia NCCL version</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t>200</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg-query -W "libcusolver*"</t>
+          <t>dpkg-query -W "libcusolver*"</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia cuSOLVER version</t>
+          <t>nVidia cuSOLVER version</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">201</t>
+          <t>201</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">grep -m1 'HPL - ' /tmp/hpl-2.3/BUGS</t>
+          <t>grep -m1 'HPL - ' /tmp/hpl-2.3/BUGS</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia HPL version</t>
+          <t>nVidia HPL version</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">202</t>
+          <t>202</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">dcgmi --version</t>
+          <t>dcgmi --version</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia DCGM management tool version</t>
+          <t>nVidia DCGM management tool version</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">203</t>
+          <t>203</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">dpkg -l | egrep -i '^(ii)\s+(cuda|nvidia-driver|nvidia-smi|nvidia-cuda-toolkit|libnccl|libcudnn|libcublas|libcusparse|libcusolver|libcufft|libcurand|libnpp|nvidia-gds|cuda-drivers)'</t>
+          <t>dpkg -l | egrep -i '^(ii)\s+(cuda|nvidia-driver|nvidia-smi|nvidia-cuda-toolkit|libnccl|libcudnn|libcublas|libcusparse|libcusolver|libcufft|libcurand|libnpp|nvidia-gds|cuda-drivers)'</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia Installed CUDA &amp; Packages List</t>
+          <t>nVidia Installed CUDA &amp; Packages List</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">204</t>
+          <t>204</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia-only</t>
+          <t>nVidia-only</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">software</t>
+          <t>software</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">nvidia-smi -</t>
+          <t>nvidia-smi -</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">nVidia CUDA GPU / Runtime Details</t>
+          <t>nVidia CUDA GPU / Runtime Details</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update benchmark workload to v1.0.22
</commit_message>
<xml_diff>
--- a/config/hw_sw_info_commands.xlsx
+++ b/config/hw_sw_info_commands.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3246,6 +3246,60 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>139.1</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>AMD, nVidia</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>git -C "${COLLECTOR_REPO_ROOT:-.}" describe --tags --always 2&gt;/dev/null || echo "no git metadata: this workload was copied, not cloned"</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Workload release (git tag of this workload repository)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>139.2</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>AMD, nVidia</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>git -C "${COLLECTOR_REPO_ROOT:-.}/.." describe --tags --always 2&gt;/dev/null || echo "not inside a cloned benchmark bundle"</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Bundle release (git tag of the bundle that holds this workload)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>